<commit_message>
Set Starter to $15, add owner brochure with first-month-free offer
- Starter raised $12 -> $15 across all docs; blended ARPU re-modeled
  ~$200 -> ~$218; financial model v2 (md + xlsx) recomputed
- $15 Starter improves the stress case (Year 3 now thinly profitable)
- New 4-page owner marketing brochure (docs/marketing/owner-brochure-mexico)
  with the launch first-month-free offer (subscription only; add-ons,
  screening, and card fees still apply)
- First-month-free offer documented in CLAUDE.md pricing; PAYG note
  added re: short 1-2 night stays with add-ons vs Airbnb
- Regenerated all affected PDFs, Word docs, and the spreadsheet

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/business/Familiar_Guest_Financial_Model_v2.xlsx
+++ b/docs/business/Familiar_Guest_Financial_Model_v2.xlsx
@@ -486,7 +486,7 @@
         <v>0.5</v>
       </c>
       <c r="C9">
-        <v>144</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10">
@@ -604,10 +604,10 @@
         <v>0.5</v>
       </c>
       <c r="C4">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="D4">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +663,7 @@
         <v/>
       </c>
       <c r="D8">
-        <v>199.5</v>
+        <v>217.5</v>
       </c>
     </row>
   </sheetData>
@@ -721,13 +721,13 @@
         <v>Blended ARPU ($)</v>
       </c>
       <c r="B4">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="C4">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="D4">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5">
@@ -735,13 +735,13 @@
         <v>Revenue ($)</v>
       </c>
       <c r="B5">
-        <v>50000</v>
+        <v>54500</v>
       </c>
       <c r="C5">
-        <v>400000</v>
+        <v>436000</v>
       </c>
       <c r="D5">
-        <v>1500000</v>
+        <v>1635000</v>
       </c>
     </row>
     <row r="6">
@@ -749,13 +749,13 @@
         <v>Gross profit (76%) ($)</v>
       </c>
       <c r="B6">
-        <v>38000</v>
+        <v>41420</v>
       </c>
       <c r="C6">
-        <v>304000</v>
+        <v>331360</v>
       </c>
       <c r="D6">
-        <v>1140000</v>
+        <v>1242600</v>
       </c>
     </row>
     <row r="7">
@@ -777,13 +777,13 @@
         <v>Operating profit ($)</v>
       </c>
       <c r="B8">
-        <v>3000</v>
+        <v>6420</v>
       </c>
       <c r="C8">
-        <v>104000</v>
+        <v>131360</v>
       </c>
       <c r="D8">
-        <v>490000</v>
+        <v>592600</v>
       </c>
     </row>
     <row r="9">
@@ -791,13 +791,13 @@
         <v>Operating margin</v>
       </c>
       <c r="B9">
-        <v>0.06</v>
+        <v>0.11779816513761468</v>
       </c>
       <c r="C9">
-        <v>0.26</v>
+        <v>0.30128440366972475</v>
       </c>
       <c r="D9">
-        <v>0.32666666666666666</v>
+        <v>0.36244648318042816</v>
       </c>
     </row>
   </sheetData>
@@ -841,13 +841,13 @@
         <v>Gross profit ($)</v>
       </c>
       <c r="B3">
-        <v>38000</v>
+        <v>41420</v>
       </c>
       <c r="C3">
-        <v>304000</v>
+        <v>331360</v>
       </c>
       <c r="D3">
-        <v>1140000</v>
+        <v>1242600</v>
       </c>
     </row>
     <row r="5">
@@ -869,13 +869,13 @@
         <v xml:space="preserve">  Operating profit ($)</v>
       </c>
       <c r="B6">
-        <v>13000</v>
+        <v>16420</v>
       </c>
       <c r="C6">
-        <v>214000</v>
+        <v>241360</v>
       </c>
       <c r="D6">
-        <v>860000</v>
+        <v>962600</v>
       </c>
     </row>
     <row r="7">
@@ -883,13 +883,13 @@
         <v xml:space="preserve">  Margin</v>
       </c>
       <c r="B7">
-        <v>0.26</v>
+        <v>0.30128440366972475</v>
       </c>
       <c r="C7">
-        <v>0.535</v>
+        <v>0.5535779816513762</v>
       </c>
       <c r="D7">
-        <v>0.5733333333333334</v>
+        <v>0.5887461773700305</v>
       </c>
     </row>
     <row r="9">
@@ -911,13 +911,13 @@
         <v xml:space="preserve">  Operating profit ($)</v>
       </c>
       <c r="B10">
-        <v>3000</v>
+        <v>6420</v>
       </c>
       <c r="C10">
-        <v>104000</v>
+        <v>131360</v>
       </c>
       <c r="D10">
-        <v>490000</v>
+        <v>592600</v>
       </c>
     </row>
     <row r="11">
@@ -925,13 +925,13 @@
         <v xml:space="preserve">  Margin</v>
       </c>
       <c r="B11">
-        <v>0.06</v>
+        <v>0.11779816513761468</v>
       </c>
       <c r="C11">
-        <v>0.26</v>
+        <v>0.30128440366972475</v>
       </c>
       <c r="D11">
-        <v>0.32666666666666666</v>
+        <v>0.36244648318042816</v>
       </c>
     </row>
     <row r="13">
@@ -953,13 +953,13 @@
         <v xml:space="preserve">  Operating profit ($)</v>
       </c>
       <c r="B14">
-        <v>-12000</v>
+        <v>-8580</v>
       </c>
       <c r="C14">
-        <v>-46000</v>
+        <v>-18640</v>
       </c>
       <c r="D14">
-        <v>-10000</v>
+        <v>92600</v>
       </c>
     </row>
     <row r="15">
@@ -967,13 +967,13 @@
         <v xml:space="preserve">  Margin</v>
       </c>
       <c r="B15">
-        <v>-0.24</v>
+        <v>-0.15743119266055045</v>
       </c>
       <c r="C15">
-        <v>-0.115</v>
+        <v>-0.04275229357798165</v>
       </c>
       <c r="D15">
-        <v>-0.006666666666666667</v>
+        <v>0.05663608562691132</v>
       </c>
     </row>
   </sheetData>
@@ -1017,13 +1017,13 @@
         <v>Subscription/commission revenue ($)</v>
       </c>
       <c r="B3">
-        <v>50000</v>
+        <v>54500</v>
       </c>
       <c r="C3">
-        <v>400000</v>
+        <v>436000</v>
       </c>
       <c r="D3">
-        <v>1500000</v>
+        <v>1635000</v>
       </c>
     </row>
     <row r="4">
@@ -1045,13 +1045,13 @@
         <v>Total revenue ($)</v>
       </c>
       <c r="B5">
-        <v>68750</v>
+        <v>73250</v>
       </c>
       <c r="C5">
-        <v>550000</v>
+        <v>586000</v>
       </c>
       <c r="D5">
-        <v>2062500</v>
+        <v>2197500</v>
       </c>
     </row>
     <row r="6">
@@ -1059,13 +1059,13 @@
         <v>Gross profit (76%) ($)</v>
       </c>
       <c r="B6">
-        <v>52250</v>
+        <v>55670</v>
       </c>
       <c r="C6">
-        <v>418000</v>
+        <v>445360</v>
       </c>
       <c r="D6">
-        <v>1567500</v>
+        <v>1670100</v>
       </c>
     </row>
     <row r="7">
@@ -1073,13 +1073,13 @@
         <v>Operating profit @ Base OpEx ($)</v>
       </c>
       <c r="B7">
-        <v>17250</v>
+        <v>20670</v>
       </c>
       <c r="C7">
-        <v>218000</v>
+        <v>245360</v>
       </c>
       <c r="D7">
-        <v>917500</v>
+        <v>1020100</v>
       </c>
     </row>
     <row r="8">
@@ -1087,13 +1087,13 @@
         <v>Operating profit @ Stress OpEx ($)</v>
       </c>
       <c r="B8">
-        <v>2250</v>
+        <v>5670</v>
       </c>
       <c r="C8">
-        <v>68000</v>
+        <v>95360</v>
       </c>
       <c r="D8">
-        <v>417500</v>
+        <v>520100</v>
       </c>
     </row>
     <row r="10">

</xml_diff>